<commit_message>
updated index to show default as T-1
</commit_message>
<xml_diff>
--- a/BSE/bse_daily.xlsx
+++ b/BSE/bse_daily.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1460"/>
+  <dimension ref="A1:E1461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39836,6 +39836,33 @@
         </is>
       </c>
     </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>16 Feb 2026</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>4919</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>29,40,812</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>82,17,71,765</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>7,505.87</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>